<commit_message>
Add QA-ready tracking plan contract
</commit_message>
<xml_diff>
--- a/files/ga4_tracking_plan_template_v2_1.xlsx
+++ b/files/ga4_tracking_plan_template_v2_1.xlsx
@@ -12,12 +12,14 @@
     <sheet name="02 Parameter Reference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03 Event Matrix" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="04 Screenshot Register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05 QA Cases" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$E$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$G$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$L$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 QA Cases'!$A$3:$K$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1042,74 +1044,74 @@
       <c r="H21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>05 QA Cases</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DebugView, GTM Preview, and network validation contract</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Analysts, developers, QA</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>One row per testable event case</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Conventions</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr"/>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Pattern / status</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Example</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Where used</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Pattern / status</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Implemented and validated</t>
+          <t>Meaning</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>Example</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Test status columns</t>
+          <t>Where used</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
@@ -1120,17 +1122,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Implemented but wrong, missing, duplicated, or using unexpected value</t>
+          <t>Implemented and validated</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1146,17 +1148,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Blocked by environment, access, consent, data, or unavailable journey</t>
+          <t>Implemented but wrong, missing, duplicated, or using unexpected value</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1172,22 +1174,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Cannot test</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Not applicable for this event</t>
+          <t>Blocked by environment, access, consent, data, or unavailable journey</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Cannot test</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Value/rule columns</t>
+          <t>Test status columns</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -1198,22 +1200,22 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>value_a | value_b</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Possible values</t>
+          <t>Not applicable for this event</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>auto | home | unknown</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Value rules</t>
+          <t>Value/rule columns</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -1221,20 +1223,20 @@
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr"/>
     </row>
-    <row r="30" ht="42" customHeight="1">
+    <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>normalized_value</t>
+          <t>value_a | value_b</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Controlled analytics values should be lowercase ASCII snake_case with accents removed</t>
+          <t>Possible values</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>pret_a_porter_femme</t>
+          <t>auto | home | unknown</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1250,22 +1252,22 @@
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ecommerce</t>
+          <t>normalized_value</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce events stay in ecommerce-only blocks and use official GA4 parameter names</t>
+          <t>Controlled analytics values should be lowercase ASCII snake_case with accents removed</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>items[].item_id</t>
+          <t>pret_a_porter_femme</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Event Matrix</t>
+          <t>Value rules</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -1273,25 +1275,25 @@
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr"/>
     </row>
-    <row r="32">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>%value%</t>
+          <t>ecommerce</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Dynamic value</t>
+          <t>Ecommerce events stay in ecommerce-only blocks and use official GA4 parameter names</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>%search_term%</t>
+          <t>items[].item_id</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Value rules/examples</t>
+          <t>Event Matrix</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -1302,22 +1304,22 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>object.key</t>
+          <t>%value%</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Nested object field</t>
+          <t>Dynamic value</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>page_data.template</t>
+          <t>%search_term%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Variable names</t>
+          <t>Value rules/examples</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -1328,28 +1330,54 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>items[].field</t>
+          <t>object.key</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Field inside each object of an array</t>
+          <t>Nested object field</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>items[].item_id</t>
+          <t>page_data.template</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ecommerce item variables</t>
+          <t>Variable names</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>items[].field</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Field inside each object of an array</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>items[].item_id</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce item variables</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1357,8 +1385,8 @@
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -6839,4 +6867,409 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>QA Cases</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Validation contract for DebugView, GTM Preview, browser network requests, and release sign-off.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>QA ID</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Journey</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Event name</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Methods</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Expected dataLayer</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Expected network / GA4 payload</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>DebugView expectation</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Evidence / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>QA-PAGE-001</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Page and content discovery</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>page_view</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>EVT-PAGE-001</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>DebugView | GTM Preview | Network</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Open the page or trigger the SPA route change once.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>page_data is available before the event; previous page_data is flushed when needed.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>GA4 event name page_view; page_location, page_title, and page_referrer are populated when available.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>One page_view appears for the initial view or route change.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Cannot test</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>QA-CONTENT-001</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Page and content discovery</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>select_content</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>EVT-CONTENT-001</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>GTM Preview | Network</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Click each consolidated content component covered by the allowed values.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>event_data.content_type, content_id, content_name, and cta_location match the clicked component.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>GA4 event name select_content; controlled values are lowercase ASCII snake_case.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>select_content appears with the selected content context.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Cannot test</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>QA-SEARCH-001</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Search and lead journey</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>EVT-SEARCH-001</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>DebugView | GTM Preview | Network</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Submit a privacy-safe search term.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>event_data.search_term is populated after PII scrubbing.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>GA4 event name search; search_term is present and contains no direct PII.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>search appears with the submitted search_term.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Cannot test</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>QA-ECOM-001</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Ecommerce journey</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>view_item_list / select_item / view_item / add_to_cart</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>EVT-ECOM-001</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>DebugView | GTM Preview | Network</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>View a product list, select an item, view detail, and add to cart when available.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>ecommerce object is flushed before each ecommerce event; items array contains required item identifiers.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>GA4 ecommerce event uses official parameters: currency/value when sent, items, items[].item_id or items[].item_name.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Each ecommerce event appears with a valid items array.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Cannot test</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>QA-PROMO-001</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Promotion journey</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>view_promotion / select_promotion</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>EVT-PROMO-001</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>GTM Preview | Network</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Expose a tracked promotion and click it.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>promotion_id, promotion_name, creative_name, creative_slot, and items are populated when available.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>GA4 event name view_promotion or select_promotion; official promotion parameters are present.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Promotion impression and click appear with matching promotion identifiers.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Cannot test</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:K8"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="J4:J208">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"KO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"Cannot test"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="J4:J208" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"OK,KO,Cannot test"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>